<commit_message>
Record USD as documented currency, drop the currency warning
All six invoices carry the $ symbol on unit prices and amounts, in the
cell number format (\$#,##0.00...) rather than the cell value, so the
earlier scan of cell values alone missed it. The currency is documented
on the invoices, not inferred, so the warning flag is removed and the
header now cites the $ formatting as its source.

Figures are unchanged: 3,258.66 kg net / 4,856.20 kg gross / 62,804 pcs
/ USD 128,225.56.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BdXXipFKSZXXT17VhbMQEJ
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Rare_Beauty_8016.xlsx
+++ b/output/HS_Code_Summary_Rare_Beauty_8016.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -861,7 +861,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>USD (na fakturách NEUVEDENA – viz kritické příznaky níže)</t>
+          <t>USD – na všech šesti fakturách uvedeno symbolem $ u jednotkových cen i částek</t>
         </is>
       </c>
       <c r="C15" s="5" t="n"/>
@@ -1058,38 +1058,28 @@
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
+          <t>Měna: USD. Na všech šesti fakturách je u jednotkových cen i u částek uveden symbol $ (formát buňky), celková částka faktury je zobrazena např. jako $10 677,40. Pro přepočet použijte celní kurz platný k datu propuštění.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
           <t>Celní hodnota = fakturovaná hodnota položek. Dodací podmínka je DDP Kněževes – při deklaraci je nutné dořešit připočitatelné/odpočitatelné náklady (přeprava a pojištění do místa vstupu do EU) dle čl. 70 a 71 celního kodexu Unie.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="18" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>KRITICKÉ PŘÍZNAKY / CRITICAL FLAGS</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>⚠ PREFERENČNÍ VĚTA – NENALEZENA</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
-      <c r="K28" s="6" t="n"/>
-    </row>
-    <row r="29" ht="58" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>V žádné ze šesti faktur (1383-01 až 1388-01) ani v HBL NENÍ uvedena preferenční věta – prohlášení o preferenčním původu podle Dohody o volném obchodu EU–Korejská republika. Doklady uvádějí pouze '* COUNTRY OF ORIGIN : Made in Korea', což preferenční původ NEPROKAZUJE. Bez preferenční věty nelze uplatnit preferenční sazbu a použije se všeobecná (třetizemní) sazba cla. Pro CN 3304 99 00 je všeobecná sazba cla 0 %, takže dopad na clo je v tomto konkrétním případě nulový (ověřte v TARIC k datu propuštění); DPH se uplatní v plné výši. DOPORUČENÍ: vyžádat od GYC Gayang Corp. doplnění preferenční věty na faktury včetně čísla povolení schváleného vývozce.</t>
         </is>
       </c>
       <c r="B29" s="5" t="n"/>
@@ -1103,27 +1093,27 @@
       <c r="J29" s="5" t="n"/>
       <c r="K29" s="6" t="n"/>
     </row>
-    <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+    <row r="30" ht="58" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>V žádné ze šesti faktur (1383-01 až 1388-01) ani v HBL NENÍ uvedena preferenční věta – prohlášení o preferenčním původu podle Dohody o volném obchodu EU–Korejská republika. Doklady uvádějí pouze '* COUNTRY OF ORIGIN : Made in Korea', což preferenční původ NEPROKAZUJE. Bez preferenční věty nelze uplatnit preferenční sazbu a použije se všeobecná (třetizemní) sazba cla. Pro CN 3304 99 00 je všeobecná sazba cla 0 %, takže dopad na clo je v tomto konkrétním případě nulový (ověřte v TARIC k datu propuštění); DPH se uplatní v plné výši. DOPORUČENÍ: vyžádat od GYC Gayang Corp. doplnění preferenční věty na faktury včetně čísla povolení schváleného vývozce.</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="5" t="n"/>
+      <c r="J30" s="5" t="n"/>
+      <c r="K30" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>CBAM – NEAPLIKUJE SE</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="n"/>
-      <c r="K31" s="6" t="n"/>
-    </row>
-    <row r="32" ht="58" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>HS 3304.99 / CN 3304 99 00 (kosmetické přípravky) NENÍ zbožím uvedeným v příloze I nařízení CBAM (cement, elektřina, hnojiva, železo a ocel, hliník, vodík). Vyhledání příjemce v registru reference/CBAM_receivers_CZ.xlsx proto není pro tuto zásilku vyžadováno. Pro úplnost bylo přesto provedeno: příjemce 'Rare Beauty' ani 'Maurice Ward &amp; Co., s.r.o.' se v registru (101 řádků) NENACHÁZÍ – pokud by tato společnost měla někdy dovážet CBAM zboží, je třeba ji do registru doplnit.</t>
         </is>
       </c>
       <c r="B32" s="5" t="n"/>
@@ -1137,27 +1127,27 @@
       <c r="J32" s="5" t="n"/>
       <c r="K32" s="6" t="n"/>
     </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
-        <is>
-          <t>⚠ MĚNA NENÍ NA FAKTURÁCH UVEDENA</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n"/>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="5" t="n"/>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="5" t="n"/>
-      <c r="I34" s="5" t="n"/>
-      <c r="J34" s="5" t="n"/>
-      <c r="K34" s="6" t="n"/>
-    </row>
-    <row r="35" ht="58" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>Všech šest faktur uvádí jednotkové ceny i částky bez označení měny. Vzhledem k tomu, že kupujícím je Rare Beauty Brands Inc. (Boston, USA), je v souhrnu použita měna USD. PŘED PODÁNÍM CELNÍHO PROHLÁŠENÍ POTVRĎTE MĚNU s odesílatelem/klientem a použijte celní kurz platný k datu propuštění.</t>
+    <row r="33" ht="58" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>HS 3304.99 / CN 3304 99 00 (kosmetické přípravky) NENÍ zbožím uvedeným v příloze I nařízení CBAM (cement, elektřina, hnojiva, železo a ocel, hliník, vodík). Vyhledání příjemce v registru reference/CBAM_receivers_CZ.xlsx proto není pro tuto zásilku vyžadováno. Pro úplnost bylo přesto provedeno: příjemce 'Rare Beauty' ani 'Maurice Ward &amp; Co., s.r.o.' se v registru (101 řádků) NENACHÁZÍ – pokud by tato společnost měla někdy dovážet CBAM zboží, je třeba ji do registru doplnit.</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n"/>
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="5" t="n"/>
+      <c r="J33" s="5" t="n"/>
+      <c r="K33" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>⚠ ROZPOR V PLATBĚ PŘEPRAVNÉHO</t>
         </is>
       </c>
       <c r="B35" s="5" t="n"/>
@@ -1171,27 +1161,27 @@
       <c r="J35" s="5" t="n"/>
       <c r="K35" s="6" t="n"/>
     </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr">
-        <is>
-          <t>⚠ ROZPOR V PLATBĚ PŘEPRAVNÉHO</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="n"/>
-      <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="5" t="n"/>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="5" t="n"/>
-      <c r="K37" s="6" t="n"/>
-    </row>
-    <row r="38" ht="58" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
+    <row r="36" ht="58" customHeight="1">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>Faktury uvádějí '* FREIGHT COLLECT', HBL KIMXHAM2608001 uvádí 'FREIGHT PREPAID AS ARRANGED'. Rozpor je nutné vyjasnit pro správné stanovení celní hodnoty (připočitatelné náklady dle čl. 71 celního kodexu Unie).</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="5" t="n"/>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="5" t="n"/>
+      <c r="I36" s="5" t="n"/>
+      <c r="J36" s="5" t="n"/>
+      <c r="K36" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t>POPIS ZBOŽÍ – ZDROJ POUZE ANGLICKY</t>
         </is>
       </c>
       <c r="B38" s="5" t="n"/>
@@ -1205,54 +1195,39 @@
       <c r="J38" s="5" t="n"/>
       <c r="K38" s="6" t="n"/>
     </row>
-    <row r="40">
-      <c r="A40" s="19" t="inlineStr">
-        <is>
-          <t>POPIS ZBOŽÍ – ZDROJ POUZE ANGLICKY</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="n"/>
-      <c r="C40" s="5" t="n"/>
-      <c r="D40" s="5" t="n"/>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="5" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="5" t="n"/>
-      <c r="I40" s="5" t="n"/>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="6" t="n"/>
-    </row>
-    <row r="41" ht="58" customHeight="1">
-      <c r="A41" s="9" t="inlineStr">
+    <row r="39" ht="58" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>V dokladech není k dispozici český popis zboží – faktury uvádějí pouze anglické názvy výrobků. Český popis ve sloupci 'Popis zboží' byl proto sestaven podle nomenklatury CN a názvů výrobků z faktur; původní anglické názvy jsou zachovány v listu 'Detail – položky'.</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n"/>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="5" t="n"/>
-      <c r="I41" s="5" t="n"/>
-      <c r="J41" s="5" t="n"/>
-      <c r="K41" s="6" t="n"/>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="5" t="n"/>
+      <c r="I39" s="5" t="n"/>
+      <c r="J39" s="5" t="n"/>
+      <c r="K39" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="A34:K34"/>
+  <mergeCells count="25">
+    <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A39:K39"/>
     <mergeCell ref="B9:K9"/>
     <mergeCell ref="A24:K24"/>
     <mergeCell ref="B15:K15"/>
     <mergeCell ref="B6:K6"/>
+    <mergeCell ref="A36:K36"/>
     <mergeCell ref="B5:K5"/>
     <mergeCell ref="B4:K4"/>
     <mergeCell ref="A25:K25"/>
-    <mergeCell ref="A41:K41"/>
     <mergeCell ref="B7:K7"/>
     <mergeCell ref="B16:K16"/>
-    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A33:K33"/>
     <mergeCell ref="B12:K12"/>
     <mergeCell ref="A32:K32"/>
     <mergeCell ref="B11:K11"/>
@@ -1263,10 +1238,7 @@
     <mergeCell ref="A29:K29"/>
     <mergeCell ref="B13:K13"/>
     <mergeCell ref="A38:K38"/>
-    <mergeCell ref="A28:K28"/>
     <mergeCell ref="B10:K10"/>
-    <mergeCell ref="A40:K40"/>
-    <mergeCell ref="A31:K31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>